<commit_message>
Excel shablonda "Correct" ustunidagi data validation'ni tuzatish (E variant qo'shilmagan edi)
E ustunini qo'shganimda (avvalgi commit) faqat katak QIYMATLARINI
o'ngga surgan edim — lekin "To'g'ri javob" ustunidagi dropdown (data
validation) o'zi ANIQ ustun manziliga (F) bog'langan bo'lib, u
avtomatik ko'chmadi. Natijada dropdown fizik jihatdan F ustunida (endi
"E javob" ustuni) qolib ketgan, "Correct" ustuni (endi G) esa
validatsiyasiz qoldi va uning ro'yxati hali ham faqat A-D edi.

Endi validatsiya to'g'ri G ustuniga (Correct) ko'chirildi, manba
ro'yxati $B$1:$F$1 (A,B,C,D,E sarlavhalari)ga kengaytirildi.
</commit_message>
<xml_diff>
--- a/src/main/resources/templates/template_For_Import.xlsx
+++ b/src/main/resources/templates/template_For_Import.xlsx
@@ -459,11 +459,11 @@
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultColWidth="31.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="5" style="2" width="31.5546875"/>
+    <col min="6" max="6" customWidth="true" style="2" width="31.5546875"/>
+    <col min="7" max="7" customWidth="true" style="2" width="31.5546875"/>
+    <col min="8" max="8" customWidth="true" style="2" width="31.5546875"/>
     <col min="9" max="16384" style="2" width="31.5546875"/>
-    <col min="8" max="8" style="2" width="31.5546875" customWidth="true"/>
-    <col min="7" max="7" style="2" width="31.5546875" customWidth="true"/>
-    <col min="1" max="5" style="2" width="31.5546875"/>
-    <col min="6" max="6" style="2" width="31.5546875" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -520,8 +520,8 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F1048576" xr:uid="{083D6D57-0722-4313-8085-287E416C26E5}">
-      <formula1>$B$1:$E$1</formula1>
+    <dataValidation type="list" sqref="G2:G1048576" allowBlank="true" errorStyle="stop" showErrorMessage="true">
+      <formula1>$B$1:$F$1</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
template_For_Import.xlsx: "Correct" ustunidagi eski (faqat bitta harf) tekshiruv olib tashlandi
Shablon faylida "Correct" ustuni Excel'ning o'z ("data validation")
ro'yxat-tekshiruvi bilan cheklangan edi (faqat A/B/C/D/E — bitta harf),
bu ko'p-to'g'ri-javobli savollar (ExcelService#parseCorrectIndexes,
"B,C" yoki "B C" formatini allaqachon qo'llab-quvvatlaydi) qo'shilishi
BILAN eskirib qolgan edi — foydalanuvchi vergul bilan bir nechta harf
kiritmoqchi bo'lganda Excel "Это значение не соответствует
ограничениям..." xatosi bilan rad etardi.

Endi cheklov olib tashlandi, sarlavha esa "Correct (B yoki B, C)" deb
o'zgartirildi — formatni jadvalning o'zida tushunarli qilib ko'rsatish
uchun (foydalanuvchi so'rovi, 2026-09-05).
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/main/resources/templates/template_For_Import.xlsx
+++ b/src/main/resources/templates/template_For_Import.xlsx
@@ -1,113 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent>
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\JavaPrograms\TestProject\src\main\resources\templates\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD02C37C-DD14-436F-B59B-D1418897F0A9}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EF2D30AB-4CB7-4913-B6BB-3CA9A4955B7A}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Лист1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лист1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="16">
-  <si>
-    <t>Question</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>D</t>
-  </si>
-  <si>
-    <t>Correct</t>
-  </si>
-  <si>
-    <t>Exceldagi test savol?</t>
-  </si>
-  <si>
-    <t>Exceldagi test javob A</t>
-  </si>
-  <si>
-    <t>Exceldagi test javob B</t>
-  </si>
-  <si>
-    <t>Exceldagi test javob C</t>
-  </si>
-  <si>
-    <t>Exceldagi test javob D</t>
-  </si>
-  <si>
-    <t>Exceldagi test comment</t>
-  </si>
-  <si>
-    <t>Comment (Faqat to'g'ri javob uchun)</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>E</t>
-  </si>
-  <si>
-    <t>Exceldagi test javob E</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
+      <name val="Calibri"/>
+      <charset val="204"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="Calibri"/>
+      <charset val="204"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -132,30 +62,89 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -455,75 +444,106 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05A55F1F-879E-4740-BE22-BEE0EF3E24DE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultColWidth="31.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="31.5546875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="5" style="2" width="31.5546875"/>
-    <col min="6" max="6" customWidth="true" style="2" width="31.5546875"/>
-    <col min="7" max="7" customWidth="true" style="2" width="31.5546875"/>
-    <col min="8" max="8" customWidth="true" style="2" width="31.5546875"/>
-    <col min="9" max="16384" style="2" width="31.5546875"/>
+    <col width="31.5546875" customWidth="1" style="2" min="1" max="5"/>
+    <col width="31.5546875" customWidth="1" style="2" min="6" max="6"/>
+    <col width="31.5546875" customWidth="1" style="2" min="7" max="7"/>
+    <col width="31.5546875" customWidth="1" style="2" min="8" max="8"/>
+    <col width="31.5546875" customWidth="1" style="2" min="9" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s" s="3">
-        <v>14</v>
-      </c>
-      <c r="G1" t="s" s="3">
-        <v>5</v>
-      </c>
-      <c r="H1" t="s" s="3">
-        <v>12</v>
+    <row r="1" ht="28.8" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Question</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Correct (B yoki B, C)</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Comment (Faqat to'g'ri javob uchun)</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="G2" t="s" s="1">
-        <v>2</v>
-      </c>
-      <c r="H2" t="s" s="1">
-        <v>11</v>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Exceldagi test savol?</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Exceldagi test javob A</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Exceldagi test javob B</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Exceldagi test javob C</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Exceldagi test javob D</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>Exceldagi test javob E</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>Exceldagi test comment</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" sqref="G2:G1048576" allowBlank="true" errorStyle="stop" showErrorMessage="true">
-      <formula1>$B$1:$F$1</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>